<commit_message>
docs: README brought up to date (28 October), outstanding tests and the old-stack retirement list; PR 11 test report; fix summary ranges in the PR 5 report
</commit_message>
<xml_diff>
--- a/Reports/PR-5-Back-Office-Language-Test-Report.xlsx
+++ b/Reports/PR-5-Back-Office-Language-Test-Report.xlsx
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Results'!E2:E306,"Passed")</f>
+        <f>COUNTIF('Test Results'!E2:E321,"Passed")</f>
         <v/>
       </c>
     </row>
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Results'!E2:E306,"Failed")</f>
+        <f>COUNTIF('Test Results'!E2:E321,"Failed")</f>
         <v/>
       </c>
     </row>
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF('Test Results'!E2:E306,"Skipped")</f>
+        <f>COUNTIF('Test Results'!E2:E321,"Skipped")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: README up to date, outstanding list, PR 11 test report (#12)
* docs: README brought up to date (28 October), outstanding tests and the old-stack retirement list; PR 11 test report; fix summary ranges in the PR 5 report

* docs: cutover progress (kando-main created, Production env switched) and what is left to decide

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Reports/PR-5-Back-Office-Language-Test-Report.xlsx
+++ b/Reports/PR-5-Back-Office-Language-Test-Report.xlsx
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Results'!E2:E306,"Passed")</f>
+        <f>COUNTIF('Test Results'!E2:E321,"Passed")</f>
         <v/>
       </c>
     </row>
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Results'!E2:E306,"Failed")</f>
+        <f>COUNTIF('Test Results'!E2:E321,"Failed")</f>
         <v/>
       </c>
     </row>
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF('Test Results'!E2:E306,"Skipped")</f>
+        <f>COUNTIF('Test Results'!E2:E321,"Skipped")</f>
         <v/>
       </c>
     </row>

</xml_diff>